<commit_message>
Update Requirements Stack Spreadsheet
</commit_message>
<xml_diff>
--- a/docs/Project 3_Requirements.xlsx
+++ b/docs/Project 3_Requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7d5ca52fbaa145f3/Desktop/EECS 581/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7d5ca52fbaa145f3/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6FBCFD9-CC05-4900-9586-D58157BF3584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA68C8C8-D8D2-489C-8948-6CB8968CF711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="14856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="12480" windowHeight="14736" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agile_Reference_Stories" sheetId="1" r:id="rId1"/>
@@ -1104,7 +1104,9 @@
       <c r="D2" s="3">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" customHeight="1">
       <c r="A3" s="3">
@@ -1119,7 +1121,9 @@
       <c r="D3" s="3">
         <v>2</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1">
       <c r="A4" s="3">
@@ -1134,7 +1138,9 @@
       <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1">
       <c r="A5" s="3">
@@ -1149,7 +1155,9 @@
       <c r="D5" s="3">
         <v>4</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="15.75" customHeight="1">
       <c r="A6" s="3">
@@ -1164,7 +1172,9 @@
       <c r="D6" s="3">
         <v>5</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1">
       <c r="A7" s="3">
@@ -1179,7 +1189,9 @@
       <c r="D7" s="3">
         <v>6</v>
       </c>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1">
       <c r="A8" s="3">
@@ -1194,7 +1206,9 @@
       <c r="D8" s="3">
         <v>7</v>
       </c>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:5" ht="15.75" customHeight="1">
       <c r="A9" s="3">

</xml_diff>